<commit_message>
fix(import): infra_costs template full headers for NocoBase (ID, serverId, provider, notes)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/import/infra_costs-import-template.xlsx
+++ b/import/infra_costs-import-template.xlsx
@@ -416,124 +416,166 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>role</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>amount</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>period</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>effectiveFrom</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>serverId</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>provider</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>bypass</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Обход · VPS (Нидерланды)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>RUB</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>890</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="G2" s="1" t="n">
         <v>46023</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>selectel</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>ID ВМ в биллинге</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>exit</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Выход · транзит</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>12</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="G3" s="1" t="n">
         <v>46023</v>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>hetzner</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>bot_aux</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Бот + NocoBase (VPS)</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Бот + NocoBase</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>RUB</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>350</v>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="G4" s="1" t="n">
         <v>46113</v>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>yandex</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(import): infra_costs column order notes before serverId/provider
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/import/infra_costs-import-template.xlsx
+++ b/import/infra_costs-import-template.xlsx
@@ -457,17 +457,17 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>serverId</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>provider</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>notes</t>
         </is>
       </c>
     </row>
@@ -498,14 +498,14 @@
       <c r="G2" s="1" t="n">
         <v>46023</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>ID ВМ в биллинге</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>selectel</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>ID ВМ в биллинге</t>
         </is>
       </c>
     </row>
@@ -536,12 +536,12 @@
       <c r="G3" s="1" t="n">
         <v>46023</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="H3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
         <is>
           <t>hetzner</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
@@ -570,12 +570,12 @@
       <c r="G4" s="1" t="n">
         <v>46113</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="H4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>yandex</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>